<commit_message>
fix(excel): resolve bulk import error by seeding participants, fixing column detection, and providing valid 6-workshop test spreadsheets
</commit_message>
<xml_diff>
--- a/SkillHub.Web/wwwroot/sample_workshops.xlsx
+++ b/SkillHub.Web/wwwroot/sample_workshops.xlsx
@@ -2,13 +2,178 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <sheets>
-    <sheet name="Workshops" sheetId="1" r:id="rId1"/>
+    <sheet name="Enrollments" sheetId="1" r:id="rId1"/>
+    <sheet name="Workshops" sheetId="2" r:id="rId2"/>
+    <sheet name="Participants" sheetId="3" r:id="rId3"/>
+    <sheet name="Instructors" sheetId="4" r:id="rId4"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:D7"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>ParticipantEmail</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>WorkshopCode</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>WorkshopTitle</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ParticipantName</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>andres.mejia@correo.com</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>FOT-001</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Fotografía Urbana y Manejo de Luz Natural</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Andrés Felipe Mejía Arango</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>rosa.barrios@correo.com</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>COC-001</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Cocina Mediterránea Básica</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Rosa Elena Barrios Polo</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>mauricio.jimenez@correo.com</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>ORA-001</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Oratoria y Comunicación Asertiva</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Mauricio Jiménez Cárdenas</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>natalia.herrera@correo.com</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>DIS-001</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Fundamentos de Diseño Visual y Branding</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Natalia Herrera Castaño</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>paola.vargas@correo.com</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>MAT-001</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Matemáticas Básicas y Aplicadas</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Paola Andrea Vargas Mora</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>jorge.perez@correo.com</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>MUS-001</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Guitarra desde cero</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Jorge Andrés Pérez Rojas</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:H7"/>
   <sheetData>
     <row r="1">
@@ -307,4 +472,643 @@
     </row>
   </sheetData>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B42"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>FullName</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Ana María Jaramillo Gaviria</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>ana.jaramillo@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Ana Martínez</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>ana.martinez@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Andrés Felipe Mejía Arango</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>andres.mejia@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Andrés Mauricio Salazar Ortiz</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>andres.salazar@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Camila Andrea Cárdenas Ruiz</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>camila.cardenas@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Carlos López</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>carlos.lopez@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Carlos Eduardo Rincón Díaz</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>carlos.rincon@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Cristian David Becerra Mejía</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>cristian.becerra@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Daniela Morales Pineda</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>daniela.morales@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Diego Alejandro Muñoz Peña</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>diego.munoz@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Esteban Rodríguez Molina</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>esteban.rodriguez@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Felipe Agudelo Marín</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>felipe.agudelo@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Hernán Darío Quintero Gil</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>hernan.quintero@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Isabella Navarro Fuentes</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>isabella.navarro@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ivan</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>ivan@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Javier Alonso Cuéllar Pardo</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>javier.cuellar@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Jorge Andrés Pérez Rojas</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>jorge.perez@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Juan Pérez</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>juan.perez@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Juan Camilo Restrepo Vélez</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>juan.restrepo@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Juliana Ortega Sánchez</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>juliana.ortega@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Kevin Stiven Mosquera Palacios</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>kevin.mosquera@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Laura Sofía Martínez Suárez</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>laura.martinez@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Luis Fernando Arias Cano</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>luis.arias@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Luz Marina Ospina Ríos</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>luz.ospina@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Manuela Escobar Toro</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>manuela.escobar@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>María Rodríguez</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>maria.rodriguez@example.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>María Fernanda Torres León</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>maria.torres@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Mariana Londoño Álvarez</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>mariana.londono@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Mauricio Jiménez Cárdenas</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>mauricio.jimenez@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Natalia Herrera Castaño</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>natalia.herrera@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Natalia Montoya Correa</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>natalia.montoya@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Óscar Iván Guerrero Lozano</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>oscar.guerrero@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>Paola Andrea Vargas Mora</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>paola.vargas@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>Paula Andrea Zapata Ríos</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>paula.zapata@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Rosa Elena Barrios Polo</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>rosa.barrios@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>Santiago Ramírez Henao</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>santiago.ramirez@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Sara Valencia Bermúdez</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>sara.valencia@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Sebastián Castro Duque</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>sebastian.castro@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>Valentina Gómez Ruiz</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>valentina.gomez@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Wilmer Alfonso Benítez Cruz</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>wilmer.benitez@correo.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>Yuliana Patiño Osorio</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>yuliana.patino@correo.com</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:C7"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>FullName</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Specialty</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Carlos Mendoza</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>carlos.mendoza@skillhub.com</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Fotografía</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Laura Gómez</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>laura.gomez@skillhub.com</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Cocina</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Andrés Torres</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>andres.torres@skillhub.com</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Oratoria</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sofía Morales</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>sofia.morales@skillhub.com</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Diseño Gráfico</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Hernán Darío Quintero Gil</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>hernan.quintero@correo.com</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Música</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Admin SkillHub</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>admin@skillhub.com</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Coordinación</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+</worksheet>
 </file>
</xml_diff>